<commit_message>
feat(desktop): add startup ping, BYOK gemini support, demo script and dojo simulator
</commit_message>
<xml_diff>
--- a/assets/catalogo_actualizado.xlsx
+++ b/assets/catalogo_actualizado.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -527,16 +527,16 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Harina 000 Cañuelas</t>
+          <t>Alfajor Guaymallén chocolate</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Bolsa 25kg</t>
+          <t>Caja x 40</t>
         </is>
       </c>
       <c r="D2" s="4" t="n">
-        <v>18500</v>
+        <v>18000</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -545,7 +545,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Harinas</t>
+          <t>Golosinas</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -562,12 +562,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Aceite de Girasol Cañuelas</t>
+          <t>Alfajor Jorgito blanco</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Caja 12x900ml</t>
+          <t>Caja x 24</t>
         </is>
       </c>
       <c r="D3" s="4" t="n">
@@ -580,7 +580,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Aceites</t>
+          <t>Golosinas</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -597,16 +597,16 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Fideos Guiseros Matarazzo</t>
+          <t>Alfajor Havanna clásico</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Fardo 10x500g</t>
+          <t>Caja x 12</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
-        <v>11200</v>
+        <v>24000</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -615,7 +615,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Pastas Secas</t>
+          <t>Golosinas</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -632,16 +632,16 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Arroz Largo Fino Lucchetti</t>
+          <t>Chocolate Milka Leger 45g</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Fardo 10x1kg</t>
+          <t>Caja x 24</t>
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>14000</v>
+        <v>28800</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
@@ -650,7 +650,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Arroces</t>
+          <t>Chocolates</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -667,16 +667,16 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Azúcar Ledesma clásica</t>
+          <t>Chicles Beldent menta</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Fardo 10x1kg</t>
+          <t>Caja x 20</t>
         </is>
       </c>
       <c r="D6" s="4" t="n">
-        <v>10290</v>
+        <v>12000</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
@@ -685,7 +685,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Endulzantes</t>
+          <t>Golosinas</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -702,16 +702,16 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Leche Entera La Serenísima</t>
+          <t>Caramelos Sugus surtidos 500g</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Caja 12x1L</t>
+          <t>Bolsa</t>
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>17400</v>
+        <v>4500</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -720,7 +720,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Lácteos</t>
+          <t>Golosinas</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -737,16 +737,16 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Yerba Playadito suave</t>
+          <t>Coca Cola 500ml</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Fardo 10x1kg</t>
+          <t>Pack x 6</t>
         </is>
       </c>
       <c r="D8" s="4" t="n">
-        <v>38000</v>
+        <v>8400</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
@@ -755,7 +755,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Infusiones</t>
+          <t>Bebidas</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -772,16 +772,16 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Cerveza Quilmes Clásica</t>
+          <t>Coca Cola 1.5L</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Cajón 12x1L</t>
+          <t>Pack x 6</t>
         </is>
       </c>
       <c r="D9" s="4" t="n">
-        <v>19500</v>
+        <v>14400</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
@@ -807,16 +807,16 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Coca Cola Original</t>
+          <t>Sprite 1.5L</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Pack 6x2.25L</t>
+          <t>Pack x 6</t>
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>16500</v>
+        <v>13800</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -842,16 +842,16 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Puré de Tomate Noel</t>
+          <t>Cerveza Quilmes clásica 473ml</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Caja 12x520g</t>
+          <t>Pack x 6</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>8900</v>
+        <v>8100</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
@@ -860,7 +860,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Conservas</t>
+          <t>Bebidas</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -877,16 +877,16 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Galletitas Criollitas</t>
+          <t>Agua mineral Villavicencio 500ml</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Caja 20x100g</t>
+          <t>Pack x 6</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>12500</v>
+        <v>5400</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -895,10 +895,150 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
+          <t>Bebidas</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>ART-012</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Papas fritas Lays clásicas 85g</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Tira x 10</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>18500</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Snacks</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>ART-013</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Galletitas Oreo 118g</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Pack x 6</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>7200</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
           <t>Galletitas</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>ART-014</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Cigarrillos Philip Morris Box 20</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Atado</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>3200</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Tabaquería</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>ART-015</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Encendedor Bic mini</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Blister x 12</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>15600</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Varios</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>General</t>
         </is>

</xml_diff>